<commit_message>
Handover sheets rebuilt on the final live snapshot: 88 held, 13 wrongly Passed
Another worker was editing the same suites during the pass and the numbers moved:
91 -> 88 held and 16 -> 13 already marked Passed, because C30074/C30075/C30082 were
checked and passed. Both figures were right for their minute; the sheets carry the
later one, stamp the read time, and say why it matters.

Every count is now computed from the snapshot rather than typed in. README records
what is complete, what is not, and the one figure not re-observed by this pass.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/handover/Manual-Tester-Handover_2026-08-12.xlsx
+++ b/build/handover/Manual-Tester-Handover_2026-08-12.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -481,7 +481,8 @@
     <row r="2" ht="120" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Release is tomorrow. This sheet is for you. It has three lists in it, one per tab, and this page explains what they are and the one rule that matters most. You do not need to know anything about how the tests were written to use it.</t>
+          <t>Release is tomorrow. This sheet is for you. It has three lists in it, one per tab, and this page explains what they are and the one rule that matters most. You do not need to know anything about how the tests were written to use it.
+Row 5 says exactly when these numbers were read, and why that matters today.</t>
         </is>
       </c>
     </row>
@@ -536,7 +537,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>This is not a formality. It has already happened. Checked in TestRail this morning: 16 tests that cannot currently be judged already have a Passed result recorded against them. A test nobody could run cannot have passed. Those 16 are listed on the last tab and marked, and they need changing to Blocked before anyone reads them as evidence that the feature works.</t>
+          <t>This is not a formality. It has already happened. Read from TestRail as this sheet was written: 13 tests that cannot currently be judged already have a Passed result recorded against them. A test nobody could run cannot have passed. They are listed on the last tab and shaded, and they need changing to Blocked before anyone reads them as evidence that the feature works.</t>
         </is>
       </c>
     </row>
@@ -555,7 +556,7 @@
         <is>
           <t>Tab 2, "Problems found, not reported". Three real faults we found and confirmed. No ticket has been raised for any of them. If you want to raise the ticket yourself, everything you need to paste in is on the row, and there is a blank column for you to write the ticket number in.
 Tab 3, "Old tickets that mislead". Four tickets where what the ticket says and what the product actually does no longer match. Three say they are closed and the fault is still there. One is still open and the fault is gone.
-Tab 4, "Tests that cannot be run yet". All 91 of them, with one plain sentence each.</t>
+Tab 4, "Tests that cannot be run yet". All 88 of them, with one plain sentence each.</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -603,9 +604,9 @@
       <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Filters: 97 to run, 18 to skip (115 in total).
-Schedule: 145 to run, 31 to skip (176 in total).
+Schedule: 148 to run, 28 to skip (176 in total).
 Report Suite: 438 to run, 42 to skip (480 in total).
-All three together: 680 to run, 91 to skip, 771 in total.</t>
+All three together: 683 to run, 88 to skip, 771 in total.</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -622,16 +623,39 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
+          <t>When these numbers were taken</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Every count and every list here was read from TestRail at 2026-08-12T05:53:56Z.
+PLEASE NOTE THE TIME, because it matters today. Another member of the team was working on the same tests while this sheet was being written, and the numbers moved twice in the hour before it was finished: three Schedule tests came off the skip list because they were checked and passed. So treat this as a photograph taken at that minute, not a permanent count. If a test on the last tab no longer says it is waiting on something when you open it, believe the test, not this sheet.</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>A count taken an hour earlier said 91 tests to skip and 16 of them wrongly marked Passed. It now says 88 and 13, because three Schedule tests were checked and passed while this was being written. Neither figure is wrong - they are different minutes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="190" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
           <t>One thing to know about dates on the tests</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Near the bottom of every test there is a line saying which build it was last checked against. On most tests that build is older than the one you will be testing on today.
 That does not make the test wrong. What a test expects comes from the written product description, not from the build - so a newer build never changes what a test should expect. What can change is the exact wording of a button or where something sits on screen.</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>So if a button is named slightly differently from what the test says, that is worth telling the QA lead, but it is not automatically a fault in the product.</t>
         </is>
@@ -673,7 +697,7 @@
     <row r="2" ht="120" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>THREE problems. All three are in Schedule. All three were seen with our own eyes on the build listed on each row, and no Jira ticket covers any of them.
+          <t>3 problems, all of them in Schedule. Every one was seen with our own eyes on the build named on its row, and no Jira ticket covers any of them.
 WHAT TO DO WITH THIS TAB: nothing, unless you want to. We were asked to hold off raising tickets, so these are written out in full in case you would rather raise them yourself. Everything you need is on the row. Use the last column to write down the ticket number if you do raise one.
 BEFORE YOU RAISE ONE, PLEASE READ THE 'What is still needed' COLUMN. Each row says what is already proven and what is still missing. A ticket that a developer can argue with costs more than no ticket at all.</t>
         </is>
@@ -1189,7 +1213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G98"/>
+  <dimension ref="A1:G95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1204,7 +1228,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Tests that cannot be run yet, and why — all 91</t>
+          <t>Tests that cannot be run yet, and why — all 88</t>
         </is>
       </c>
     </row>
@@ -1213,7 +1237,7 @@
         <is>
           <t>Mark every test on this tab BLOCKED. Do not mark any of them Passed.
 Each row says in one plain sentence what the test is waiting on. The same sentence is on the test itself, at the bottom of its Expected Results.
-TWO THINGS TO LOOK AT FIRST. (1) The column 'Already has a result?' - 16 of these tests already say Passed in the test run. Those need changing to Blocked; they are the most useful thing on this tab. (2) 14 Schedule tests are all waiting on the same one thing - a second login that is not an administrator. One login would release all 14 at once.
+TWO THINGS TO LOOK AT FIRST. (1) The column 'Already has a result?' - 13 of these tests already say Passed in the test run, and they are shaded. Those need changing to Blocked; they are the most useful thing on this tab. (2) 11 Schedule tests are all waiting on the same one thing - a second login that is not an administrator. One login would release them all at once.
 The 'What it is waiting on' wording is quoted from the test itself, so it matches what you will read on the case. The only thing changed is that document reference codes have been spelled out as 'the written description'.</t>
         </is>
       </c>
@@ -1901,7 +1925,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>SCHEDULE — 31 TESTS TO SKIP</t>
+          <t>SCHEDULE — 28 TESTS TO SKIP</t>
         </is>
       </c>
       <c r="B24" s="5" t="n"/>
@@ -2112,7 +2136,7 @@
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>needs a second sign-in as a user with no staff record of their own</t>
+          <t>point 4 needs a user with no staff record of their own; points 1 to 3 are observed and pass</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -2132,22 +2156,22 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>C30074</t>
+          <t>C30076</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30074</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30076</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>Schedule: View grants the full read-only experience across the whole page</t>
+          <t>With Schedule: View OFF, the Schedule top-level nav item is hidden entirely</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>needs a second sign-in as a view-only user</t>
+          <t>needs a second sign-in as a user without the Schedule permission</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -2167,22 +2191,22 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>C30075</t>
+          <t>C30077</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30075</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30077</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>View-only: every editing affordance is hidden or disabled</t>
+          <t>Schedule: Edit unlocks all creation and modification interactions</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>needs a second sign-in as a view-only user</t>
+          <t>needs a second sign-in as an edit-without-delete user</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -2202,22 +2226,22 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>C30076</t>
+          <t>C30078</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30076</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30078</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>With Schedule: View OFF, the Schedule top-level nav item is hidden entirely</t>
+          <t>Edit without Delete: the user can create and modify but not remove</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>needs a second sign-in as a user without the Schedule permission</t>
+          <t>needs a second sign-in as an edit-without-delete user</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -2237,22 +2261,22 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>C30077</t>
+          <t>C30079</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30077</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30079</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>Schedule: Edit unlocks all creation and modification interactions</t>
+          <t>Schedule: Delete unlocks deleting shifts and events</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>needs a second sign-in as an edit-without-delete user</t>
+          <t>needs a second sign-in as a delete-capable user</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2272,22 +2296,22 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>C30078</t>
+          <t>C30081</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30078</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30081</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>Edit without Delete: the user can create and modify but not remove</t>
+          <t>Schedule without Work Orders: View - the sidebar hides the work order list</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>needs a second sign-in as an edit-without-delete user</t>
+          <t>needs a second sign-in as a user who cannot see work orders</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -2297,107 +2321,107 @@
       </c>
     </row>
     <row r="36" ht="46" customHeight="1">
-      <c r="A36" s="7" t="n">
+      <c r="A36" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="B36" s="7" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>Schedule</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
-        <is>
-          <t>C30079</t>
-        </is>
-      </c>
-      <c r="D36" s="7" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30079</t>
-        </is>
-      </c>
-      <c r="E36" s="7" t="inlineStr">
-        <is>
-          <t>Schedule: Delete unlocks deleting shifts and events</t>
-        </is>
-      </c>
-      <c r="F36" s="7" t="inlineStr">
-        <is>
-          <t>needs a second sign-in as a delete-capable user</t>
-        </is>
-      </c>
-      <c r="G36" s="7" t="inlineStr">
-        <is>
-          <t>Passed</t>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>C30084</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30084</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Clocking into line tasks is gated by the staff 'Time Clock' setting</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>needs a second sign-in as each of the two staff members</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>Untested</t>
         </is>
       </c>
     </row>
     <row r="37" ht="46" customHeight="1">
-      <c r="A37" s="7" t="n">
+      <c r="A37" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>Schedule</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
-        <is>
-          <t>C30081</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30081</t>
-        </is>
-      </c>
-      <c r="E37" s="7" t="inlineStr">
-        <is>
-          <t>Schedule without Work Orders: View - the sidebar hides the work order list</t>
-        </is>
-      </c>
-      <c r="F37" s="7" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>C30089</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30089</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>Shop closures do NOT block spread in V1 - shifts can land on closure days</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>waiting on the product owner's answer, and the shop-closure setting does not exist in the build</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>Untested</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="46" customHeight="1">
+      <c r="A38" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Schedule</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>C30614</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30614</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>With Work Orders: View OFF, work order details on shifts are hidden</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
         <is>
           <t>needs a second sign-in as a user who cannot see work orders</t>
         </is>
       </c>
-      <c r="G37" s="7" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="46" customHeight="1">
-      <c r="A38" s="7" t="n">
-        <v>32</v>
-      </c>
-      <c r="B38" s="7" t="inlineStr">
-        <is>
-          <t>Schedule</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>C30082</t>
-        </is>
-      </c>
-      <c r="D38" s="7" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30082</t>
-        </is>
-      </c>
-      <c r="E38" s="7" t="inlineStr">
-        <is>
-          <t>No own-only restriction: a View user sees ALL technicians' shifts</t>
-        </is>
-      </c>
-      <c r="F38" s="7" t="inlineStr">
-        <is>
-          <t>needs a second sign-in as a view-only technician</t>
-        </is>
-      </c>
-      <c r="G38" s="7" t="inlineStr">
-        <is>
-          <t>Passed</t>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
     </row>
@@ -2412,27 +2436,27 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>C30084</t>
+          <t>C38867</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30084</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/38867</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>Clocking into line tasks is gated by the staff 'Time Clock' setting</t>
+          <t>Shifts and events created before the Schedule rewrite still appear after it</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>needs a second sign-in as each of the two staff members</t>
+          <t>cannot be run now - it needs shifts noted BEFORE the release, and the release is already deployed</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>Untested</t>
+          <t>no result recorded — leave it, or mark Blocked</t>
         </is>
       </c>
     </row>
@@ -2447,27 +2471,27 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>C30089</t>
+          <t>C38868</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30089</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/38868</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>Shop closures do NOT block spread in V1 - shifts can land on closure days</t>
+          <t>Dashboard shows one schedule row per work order even with many shifts</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>waiting on the product owner's answer, and the shop-closure setting does not exist in the build</t>
+          <t>the Dashboard section this test needs does not exist in the build</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>Untested</t>
+          <t>no result recorded — leave it, or mark Blocked</t>
         </is>
       </c>
     </row>
@@ -2482,27 +2506,27 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>C30614</t>
+          <t>C38869</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30614</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/38869</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>With Work Orders: View OFF, work order details on shifts are hidden</t>
+          <t>A work order created with an appointment shows up on the Schedule board</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>needs a second sign-in as a user who cannot see work orders</t>
+          <t>work order creation offers no appointment in the build</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>no result recorded — leave it, or mark Blocked</t>
         </is>
       </c>
     </row>
@@ -2517,22 +2541,22 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>C38867</t>
+          <t>C38871</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/38867</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/38871</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>Shifts and events created before the Schedule rewrite still appear after it</t>
+          <t>Work order form offers a Priority (High/Medium/Low) that drives the sidebar</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>cannot be run now - it needs shifts noted BEFORE the release, and the release is already deployed</t>
+          <t>the Priority field this test needs does not exist in the build</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
@@ -2552,22 +2576,22 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>C38868</t>
+          <t>C38872</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/38868</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/38872</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>Dashboard shows one schedule row per work order even with many shifts</t>
+          <t>API - Schedule reads need View; writes need Edit; deletes need Delete (403)</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>the Dashboard section this test needs does not exist in the build</t>
+          <t>points 1 and 3 need a user with no Schedule permission and a user with Schedule Edit but not Delete; point 2 is observed and passes</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
@@ -2587,22 +2611,22 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>C38869</t>
+          <t>C38874</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/38869</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/38874</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>A work order created with an appointment shows up on the Schedule board</t>
+          <t>API - No pricing fields in Schedule responses; WO details need Work Orders View</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>work order creation offers no appointment in the build</t>
+          <t>point 2 needs a user without Work Orders View; point 1 is observed and passes</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -2622,22 +2646,22 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>C38871</t>
+          <t>C38926</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/38871</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/38926</t>
         </is>
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>Work order form offers a Priority (High/Medium/Low) that drives the sidebar</t>
+          <t>Default roles start at the Schedule level the spec names (view-only vs edit)</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>the Priority field this test needs does not exist in the build</t>
+          <t>needs a second sign-in as a holder of each permission level</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
@@ -2657,22 +2681,22 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>C38872</t>
+          <t>C43555</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/38872</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/43555</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>API - Schedule reads need View; writes need Edit; deletes need Delete (403)</t>
+          <t>Month view: dragging a work order onto a day creates a shift for that day</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>needs three separate sign-ins, one per permission level</t>
+          <t>waiting on the product owner's answer, and the question has not been sent yet</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
@@ -2692,22 +2716,22 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>C38874</t>
+          <t>C43582</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/38874</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/43582</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>API - No pricing fields in Schedule responses; WO details need Work Orders View</t>
+          <t>Panel button sits left of Today and its tooltip names what it will do</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>needs a second sign-in as a user who cannot see work orders</t>
+          <t>the panel button does not exist in this build</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">
@@ -2727,27 +2751,27 @@
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>C38926</t>
+          <t>C43583</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/38926</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/43583</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>Default roles start at the Schedule level the spec names (view-only vs edit)</t>
+          <t>Panel button hides the left panel and the grid widens into the space</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>needs a second sign-in as a holder of each permission level</t>
+          <t>the panel button does not exist in this build</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>no result recorded — leave it, or mark Blocked</t>
+          <t>Failed</t>
         </is>
       </c>
     </row>
@@ -2762,22 +2786,22 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>C43555</t>
+          <t>C43584</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/43555</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/43584</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>Month view: dragging a work order onto a day creates a shift for that day</t>
+          <t>What you had set up in the left panel survives hiding and showing it</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr">
         <is>
-          <t>waiting on the product owner's answer, and the question has not been sent yet</t>
+          <t>the panel button does not exist in this build</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr">
@@ -2797,17 +2821,17 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>C43582</t>
+          <t>C43585</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/43582</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/43585</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>Panel button sits left of Today and its tooltip names what it will do</t>
+          <t>On a narrow window the panel button still works and your choice holds</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
@@ -2832,17 +2856,17 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>C43583</t>
+          <t>C43586</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/43583</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/43586</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>Panel button hides the left panel and the grid widens into the space</t>
+          <t>Menus and pop-up windows reposition when the left panel is hidden</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
@@ -2852,7 +2876,7 @@
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>no result recorded — leave it, or mark Blocked</t>
         </is>
       </c>
     </row>
@@ -2867,17 +2891,17 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>C43584</t>
+          <t>C43587</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/43584</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/43587</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>What you had set up in the left panel survives hiding and showing it</t>
+          <t>Hiding the panel lasts for the rest of your sign-in but is not saved</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
@@ -2891,123 +2915,123 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="46" customHeight="1">
-      <c r="A53" s="6" t="n">
-        <v>47</v>
-      </c>
-      <c r="B53" s="6" t="inlineStr">
-        <is>
-          <t>Schedule</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="inlineStr">
-        <is>
-          <t>C43585</t>
-        </is>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/43585</t>
-        </is>
-      </c>
-      <c r="E53" s="6" t="inlineStr">
-        <is>
-          <t>On a narrow window the panel button still works and your choice holds</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
-          <t>the panel button does not exist in this build</t>
-        </is>
-      </c>
-      <c r="G53" s="6" t="inlineStr">
-        <is>
-          <t>no result recorded — leave it, or mark Blocked</t>
-        </is>
-      </c>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>REPORT SUITE — 42 TESTS TO SKIP</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n"/>
+      <c r="C53" s="5" t="n"/>
+      <c r="D53" s="5" t="n"/>
+      <c r="E53" s="5" t="n"/>
+      <c r="F53" s="5" t="n"/>
+      <c r="G53" s="5" t="n"/>
     </row>
     <row r="54" ht="46" customHeight="1">
       <c r="A54" s="6" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>Schedule</t>
+          <t>Report Suite</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>C43586</t>
+          <t>C30100</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/43586</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30100</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>Menus and pop-up windows reposition when the left panel is hidden</t>
+          <t>Opening an invoice you lack permission for shows access-denied; back works</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>the panel button does not exist in this build</t>
+          <t>waiting on one answer from the product owner about whether this person is given a link at all</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>no result recorded — leave it, or mark Blocked</t>
+          <t>Untested</t>
         </is>
       </c>
     </row>
     <row r="55" ht="46" customHeight="1">
       <c r="A55" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>C30104</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30104</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>Building a custom range on the calendar cannot exceed a 366-day span</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>the calendar cannot be driven past the 366-day span from this harness; the back end refuses a wider range but the on-screen prevention was not seen</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>Untested</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="46" customHeight="1">
+      <c r="A56" s="6" t="n">
         <v>49</v>
       </c>
-      <c r="B55" s="6" t="inlineStr">
-        <is>
-          <t>Schedule</t>
-        </is>
-      </c>
-      <c r="C55" s="6" t="inlineStr">
-        <is>
-          <t>C43587</t>
-        </is>
-      </c>
-      <c r="D55" s="6" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/43587</t>
-        </is>
-      </c>
-      <c r="E55" s="6" t="inlineStr">
-        <is>
-          <t>Hiding the panel lasts for the rest of your sign-in but is not saved</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="inlineStr">
-        <is>
-          <t>the panel button does not exist in this build</t>
-        </is>
-      </c>
-      <c r="G55" s="6" t="inlineStr">
-        <is>
-          <t>no result recorded — leave it, or mark Blocked</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="4" t="inlineStr">
-        <is>
-          <t>REPORT SUITE — 42 TESTS TO SKIP</t>
-        </is>
-      </c>
-      <c r="B56" s="5" t="n"/>
-      <c r="C56" s="5" t="n"/>
-      <c r="D56" s="5" t="n"/>
-      <c r="E56" s="5" t="n"/>
-      <c r="F56" s="5" t="n"/>
-      <c r="G56" s="5" t="n"/>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>C30131</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30131</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>A service (S) invoice with no vehicle also lands in the Parts Sales bucket</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>this organisation has no service invoice without a vehicle, so nothing lands in the Parts Sales bucket from the service side</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>Untested</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="46" customHeight="1">
       <c r="A57" s="6" t="n">
@@ -3020,22 +3044,22 @@
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>C30100</t>
+          <t>C30132</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30100</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30132</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t>Opening an invoice you lack permission for shows access-denied; back works</t>
+          <t>Reversed and voided invoices are excluded from every row; count and total</t>
         </is>
       </c>
       <c r="F57" s="6" t="inlineStr">
         <is>
-          <t>waiting on one answer from the product owner about whether this person is given a link at all</t>
+          <t>this organisation has no reversed or voided invoice inside the report date range</t>
         </is>
       </c>
       <c r="G57" s="6" t="inlineStr">
@@ -3055,22 +3079,22 @@
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>C30104</t>
+          <t>C30137</t>
         </is>
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30104</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30137</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>Building a custom range on the calendar cannot exceed a 366-day span</t>
+          <t>Duplicate asset labels get stable (#1)/(#2) suffixes that survive reloads</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>the calendar cannot be driven past the 366-day span from this harness; the back end refuses a wider range but the on-screen prevention was not seen</t>
+          <t>no customer in this organisation has two assets that produce the same label, so the numbered suffix cannot appear</t>
         </is>
       </c>
       <c r="G58" s="6" t="inlineStr">
@@ -3090,22 +3114,22 @@
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>C30131</t>
+          <t>C30141</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30131</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30141</t>
         </is>
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t>A service (S) invoice with no vehicle also lands in the Parts Sales bucket</t>
+          <t>An invoice deleted after load shows the not-found state and back returns</t>
         </is>
       </c>
       <c r="F59" s="6" t="inlineStr">
         <is>
-          <t>this organisation has no service invoice without a vehicle, so nothing lands in the Parts Sales bucket from the service side</t>
+          <t>deleting a real invoice while the report is open is not something to do on a shared environment</t>
         </is>
       </c>
       <c r="G59" s="6" t="inlineStr">
@@ -3125,22 +3149,22 @@
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>C30132</t>
+          <t>C30184</t>
         </is>
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30132</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30184</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t>Reversed and voided invoices are excluded from every row; count and total</t>
+          <t>A failed data fetch shows the error toast which fades after 5 seconds</t>
         </is>
       </c>
       <c r="F60" s="6" t="inlineStr">
         <is>
-          <t>this organisation has no reversed or voided invoice inside the report date range</t>
+          <t>a failing data fetch cannot be forced from the application</t>
         </is>
       </c>
       <c r="G60" s="6" t="inlineStr">
@@ -3160,22 +3184,22 @@
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>C30137</t>
+          <t>C30202</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30137</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30202</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>Duplicate asset labels get stable (#1)/(#2) suffixes that survive reloads</t>
+          <t>A Custom range uses the date-picker and holds a 366-day maximum span</t>
         </is>
       </c>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>no customer in this organisation has two assets that produce the same label, so the numbered suffix cannot appear</t>
+          <t>needs the calendar driven past a 366-day span, which this harness could not do</t>
         </is>
       </c>
       <c r="G61" s="6" t="inlineStr">
@@ -3195,22 +3219,22 @@
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>C30141</t>
+          <t>C30310</t>
         </is>
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30141</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30310</t>
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t>An invoice deleted after load shows the not-found state and back returns</t>
+          <t>Sales Representative selector shows on WO and Part Sale, not on imported</t>
         </is>
       </c>
       <c r="F62" s="6" t="inlineStr">
         <is>
-          <t>deleting a real invoice while the report is open is not something to do on a shared environment</t>
+          <t>waiting on an answer from the product owner</t>
         </is>
       </c>
       <c r="G62" s="6" t="inlineStr">
@@ -3230,22 +3254,22 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>C30184</t>
+          <t>C30311</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30184</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30311</t>
         </is>
       </c>
       <c r="E63" s="6" t="inlineStr">
         <is>
-          <t>A failed data fetch shows the error toast which fades after 5 seconds</t>
+          <t>Selector offers only reps whose sales-representative toggle is on</t>
         </is>
       </c>
       <c r="F63" s="6" t="inlineStr">
         <is>
-          <t>a failing data fetch cannot be forced from the application</t>
+          <t>this part of the report is not built yet</t>
         </is>
       </c>
       <c r="G63" s="6" t="inlineStr">
@@ -3265,22 +3289,22 @@
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>C30202</t>
+          <t>C30315</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30202</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30315</t>
         </is>
       </c>
       <c r="E64" s="6" t="inlineStr">
         <is>
-          <t>A Custom range uses the date-picker and holds a 366-day maximum span</t>
+          <t>Customer record shows a "Sales Representative" row; "Unassigned" when none</t>
         </is>
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>needs the calendar driven past a 366-day span, which this harness could not do</t>
+          <t>waiting on an answer from the product owner</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr">
@@ -3300,22 +3324,22 @@
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>C30310</t>
+          <t>C30372</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30310</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30372</t>
         </is>
       </c>
       <c r="E65" s="6" t="inlineStr">
         <is>
-          <t>Sales Representative selector shows on WO and Part Sale, not on imported</t>
+          <t>Core parts are excluded from both the inventory and special-order result sets</t>
         </is>
       </c>
       <c r="F65" s="6" t="inlineStr">
         <is>
-          <t>waiting on an answer from the product owner</t>
+          <t>no part in this organisation carries the core flag, so core exclusion cannot be exercised</t>
         </is>
       </c>
       <c r="G65" s="6" t="inlineStr">
@@ -3335,22 +3359,22 @@
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>C30311</t>
+          <t>C30398</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30311</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30398</t>
         </is>
       </c>
       <c r="E66" s="6" t="inlineStr">
         <is>
-          <t>Selector offers only reps whose sales-representative toggle is on</t>
+          <t>Without reports access Technician Utilization is hidden</t>
         </is>
       </c>
       <c r="F66" s="6" t="inlineStr">
         <is>
-          <t>this part of the report is not built yet</t>
+          <t>needs a second sign-in as a user without reports access, and there is one shared sign-in on this environment</t>
         </is>
       </c>
       <c r="G66" s="6" t="inlineStr">
@@ -3370,22 +3394,22 @@
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>C30315</t>
+          <t>C30407</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30315</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30407</t>
         </is>
       </c>
       <c r="E67" s="6" t="inlineStr">
         <is>
-          <t>Customer record shows a "Sales Representative" row; "Unassigned" when none</t>
+          <t>Internal hours with no default labor rate anywhere show an em-dash</t>
         </is>
       </c>
       <c r="F67" s="6" t="inlineStr">
         <is>
-          <t>waiting on an answer from the product owner</t>
+          <t>no location on this environment is set up without a default labor rate, so the em-dash state cannot be produced</t>
         </is>
       </c>
       <c r="G67" s="6" t="inlineStr">
@@ -3405,22 +3429,22 @@
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>C30372</t>
+          <t>C30408</t>
         </is>
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30372</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30408</t>
         </is>
       </c>
       <c r="E68" s="6" t="inlineStr">
         <is>
-          <t>Core parts are excluded from both the inventory and special-order result sets</t>
+          <t>Internal hours split across rated and unrated locations show a part value</t>
         </is>
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>no part in this organisation carries the core flag, so core exclusion cannot be exercised</t>
+          <t>no location on this environment is set up without a default labor rate, so a part-valued row cannot be produced</t>
         </is>
       </c>
       <c r="G68" s="6" t="inlineStr">
@@ -3440,22 +3464,22 @@
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>C30398</t>
+          <t>C30413</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30398</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30413</t>
         </is>
       </c>
       <c r="E69" s="6" t="inlineStr">
         <is>
-          <t>Without reports access Technician Utilization is hidden</t>
+          <t>Sorting Est. Lost Labor keeps em-dash rows last both ways; $0.00 sorts as 0</t>
         </is>
       </c>
       <c r="F69" s="6" t="inlineStr">
         <is>
-          <t>needs a second sign-in as a user without reports access, and there is one shared sign-in on this environment</t>
+          <t>no technician on this environment has an em-dash in Est. Lost Labor, because both locations have a default labor rate</t>
         </is>
       </c>
       <c r="G69" s="6" t="inlineStr">
@@ -3475,22 +3499,22 @@
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>C30407</t>
+          <t>C30431</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30407</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30431</t>
         </is>
       </c>
       <c r="E70" s="6" t="inlineStr">
         <is>
-          <t>Internal hours with no default labor rate anywhere show an em-dash</t>
+          <t>Reconcile exception (a): an open clock is snapshotted at each load instant</t>
         </is>
       </c>
       <c r="F70" s="6" t="inlineStr">
         <is>
-          <t>no location on this environment is set up without a default labor rate, so the em-dash state cannot be produced</t>
+          <t>needs a technician clocked in at the moment of the test, and no technician on this environment is currently clocked in</t>
         </is>
       </c>
       <c r="G70" s="6" t="inlineStr">
@@ -3510,22 +3534,22 @@
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>C30408</t>
+          <t>C30446</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30408</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30446</t>
         </is>
       </c>
       <c r="E71" s="6" t="inlineStr">
         <is>
-          <t>Internal hours split across rated and unrated locations show a part value</t>
+          <t>Technician Utilization: Location filter hidden for a one-location user</t>
         </is>
       </c>
       <c r="F71" s="6" t="inlineStr">
         <is>
-          <t>no location on this environment is set up without a default labor rate, so a part-valued row cannot be produced</t>
+          <t>needs a second sign-in as a user who can reach only one location, and there is one shared sign-in on this environment</t>
         </is>
       </c>
       <c r="G71" s="6" t="inlineStr">
@@ -3535,37 +3559,37 @@
       </c>
     </row>
     <row r="72" ht="46" customHeight="1">
-      <c r="A72" s="6" t="n">
+      <c r="A72" s="7" t="n">
         <v>65</v>
       </c>
-      <c r="B72" s="6" t="inlineStr">
+      <c r="B72" s="7" t="inlineStr">
         <is>
           <t>Report Suite</t>
         </is>
       </c>
-      <c r="C72" s="6" t="inlineStr">
-        <is>
-          <t>C30413</t>
-        </is>
-      </c>
-      <c r="D72" s="6" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30413</t>
-        </is>
-      </c>
-      <c r="E72" s="6" t="inlineStr">
-        <is>
-          <t>Sorting Est. Lost Labor keeps em-dash rows last both ways; $0.00 sorts as 0</t>
-        </is>
-      </c>
-      <c r="F72" s="6" t="inlineStr">
-        <is>
-          <t>no technician on this environment has an em-dash in Est. Lost Labor, because both locations have a default labor rate</t>
-        </is>
-      </c>
-      <c r="G72" s="6" t="inlineStr">
-        <is>
-          <t>Untested</t>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>C30458</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30458</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>Each qualifying work order appears exactly once in exactly one tab</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>the specification states two different tab-placement rules (whole work order by status, or per line state) and the product owner has been asked which governs</t>
+        </is>
+      </c>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
     </row>
@@ -3580,22 +3604,22 @@
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>C30431</t>
+          <t>C30462</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30431</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30462</t>
         </is>
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
-          <t>Reconcile exception (a): an open clock is snapshotted at each load instant</t>
+          <t>Status-to-tab mapping: Estimate, Complete, In Progress and Review work orders</t>
         </is>
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>needs a technician clocked in at the moment of the test, and no technician on this environment is currently clocked in</t>
+          <t>the specification states two different tab-placement rules (whole work order by status, or per line state) and the product owner has been asked which governs</t>
         </is>
       </c>
       <c r="G73" s="6" t="inlineStr">
@@ -3615,22 +3639,22 @@
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>C30446</t>
+          <t>C30464</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30446</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30464</t>
         </is>
       </c>
       <c r="E74" s="6" t="inlineStr">
         <is>
-          <t>Technician Utilization: Location filter hidden for a one-location user</t>
+          <t>Approved started-boundary: time or part received vs neither decides the tab</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>needs a second sign-in as a user who can reach only one location, and there is one shared sign-in on this environment</t>
+          <t>the specification states two different tab-placement rules (whole work order by status, or per line state) and the product owner has been asked which governs</t>
         </is>
       </c>
       <c r="G74" s="6" t="inlineStr">
@@ -3640,37 +3664,37 @@
       </c>
     </row>
     <row r="75" ht="46" customHeight="1">
-      <c r="A75" s="7" t="n">
+      <c r="A75" s="6" t="n">
         <v>68</v>
       </c>
-      <c r="B75" s="7" t="inlineStr">
+      <c r="B75" s="6" t="inlineStr">
         <is>
           <t>Report Suite</t>
         </is>
       </c>
-      <c r="C75" s="7" t="inlineStr">
-        <is>
-          <t>C30458</t>
-        </is>
-      </c>
-      <c r="D75" s="7" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30458</t>
-        </is>
-      </c>
-      <c r="E75" s="7" t="inlineStr">
-        <is>
-          <t>Each qualifying work order appears exactly once in exactly one tab</t>
-        </is>
-      </c>
-      <c r="F75" s="7" t="inlineStr">
-        <is>
-          <t>the specification states two different tab-placement rules (whole work order by status, or per line state) and the product owner has been asked which governs</t>
-        </is>
-      </c>
-      <c r="G75" s="7" t="inlineStr">
-        <is>
-          <t>Passed</t>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>C30467</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30467</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="inlineStr">
+        <is>
+          <t>First visit shows the default columns; the rest are in the column selector</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>the build does not follow the ratified Location rule; the defect is written up in DEFECTS-FOR-PERMISSION.md and needs the QA lead's permission before a ticket exists to point at</t>
+        </is>
+      </c>
+      <c r="G75" s="6" t="inlineStr">
+        <is>
+          <t>Untested</t>
         </is>
       </c>
     </row>
@@ -3685,22 +3709,22 @@
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>C30462</t>
+          <t>C30528</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30462</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30528</t>
         </is>
       </c>
       <c r="E76" s="6" t="inlineStr">
         <is>
-          <t>Status-to-tab mapping: Estimate, Complete, In Progress and Review work orders</t>
+          <t>Nightly snapshot records one row per then-open job per calendar date</t>
         </is>
       </c>
       <c r="F76" s="6" t="inlineStr">
         <is>
-          <t>the specification states two different tab-placement rules (whole work order by status, or per line state) and the product owner has been asked which governs</t>
+          <t>the nightly capture is written by a background process and nothing in the product reads it back in this version</t>
         </is>
       </c>
       <c r="G76" s="6" t="inlineStr">
@@ -3720,22 +3744,22 @@
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>C30464</t>
+          <t>C30530</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30464</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30530</t>
         </is>
       </c>
       <c r="E77" s="6" t="inlineStr">
         <is>
-          <t>Approved started-boundary: time or part received vs neither decides the tab</t>
+          <t>Captured Earned and Remaining use the same maths as the on-screen report</t>
         </is>
       </c>
       <c r="F77" s="6" t="inlineStr">
         <is>
-          <t>the specification states two different tab-placement rules (whole work order by status, or per line state) and the product owner has been asked which governs</t>
+          <t>the nightly capture is written by a background process and nothing in the product reads it back in this version</t>
         </is>
       </c>
       <c r="G77" s="6" t="inlineStr">
@@ -3755,22 +3779,22 @@
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>C30467</t>
+          <t>C30531</t>
         </is>
       </c>
       <c r="D78" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30467</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30531</t>
         </is>
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
-          <t>First visit shows the default columns; the rest are in the column selector</t>
+          <t>Nightly snapshot spans every location with no user location filter</t>
         </is>
       </c>
       <c r="F78" s="6" t="inlineStr">
         <is>
-          <t>the build does not follow the ratified Location rule; the defect is written up in DEFECTS-FOR-PERMISSION.md and needs the QA lead's permission before a ticket exists to point at</t>
+          <t>the nightly capture is written by a background process and nothing in the product reads it back in this version</t>
         </is>
       </c>
       <c r="G78" s="6" t="inlineStr">
@@ -3790,17 +3814,17 @@
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>C30528</t>
+          <t>C30533</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30528</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30533</t>
         </is>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>Nightly snapshot records one row per then-open job per calendar date</t>
+          <t>Nightly snapshot: a job with nothing approved is captured at $0.00; not skipped</t>
         </is>
       </c>
       <c r="F79" s="6" t="inlineStr">
@@ -3825,22 +3849,22 @@
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>C30530</t>
+          <t>C30547</t>
         </is>
       </c>
       <c r="D80" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30530</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30547</t>
         </is>
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
-          <t>Captured Earned and Remaining use the same maths as the on-screen report</t>
+          <t>With no fixed sell price and no category, Unit Sell equals Unit Cost</t>
         </is>
       </c>
       <c r="F80" s="6" t="inlineStr">
         <is>
-          <t>the nightly capture is written by a background process and nothing in the product reads it back in this version</t>
+          <t>a part cannot be saved without a category on this build, so the no-category path cannot be produced</t>
         </is>
       </c>
       <c r="G80" s="6" t="inlineStr">
@@ -3860,22 +3884,22 @@
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>C30531</t>
+          <t>C30577</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30531</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30577</t>
         </is>
       </c>
       <c r="E81" s="6" t="inlineStr">
         <is>
-          <t>Nightly snapshot spans every location with no user location filter</t>
+          <t>Inventory Value: the Location filter is hidden for a one-location user</t>
         </is>
       </c>
       <c r="F81" s="6" t="inlineStr">
         <is>
-          <t>the nightly capture is written by a background process and nothing in the product reads it back in this version</t>
+          <t>needs a second sign-in as a user with access to only one location</t>
         </is>
       </c>
       <c r="G81" s="6" t="inlineStr">
@@ -3895,22 +3919,22 @@
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>C30533</t>
+          <t>C30603</t>
         </is>
       </c>
       <c r="D82" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30533</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30603</t>
         </is>
       </c>
       <c r="E82" s="6" t="inlineStr">
         <is>
-          <t>Nightly snapshot: a job with nothing approved is captured at $0.00; not skipped</t>
+          <t>A user with ordinary reports access can open Inventory Value</t>
         </is>
       </c>
       <c r="F82" s="6" t="inlineStr">
         <is>
-          <t>the nightly capture is written by a background process and nothing in the product reads it back in this version</t>
+          <t>needs a second sign-in as a user holding only the ordinary reports access</t>
         </is>
       </c>
       <c r="G82" s="6" t="inlineStr">
@@ -3930,22 +3954,22 @@
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>C30547</t>
+          <t>C30604</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30547</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30604</t>
         </is>
       </c>
       <c r="E83" s="6" t="inlineStr">
         <is>
-          <t>With no fixed sell price and no category, Unit Sell equals Unit Cost</t>
+          <t>Without reports access Inventory Value is absent from the navigation</t>
         </is>
       </c>
       <c r="F83" s="6" t="inlineStr">
         <is>
-          <t>a part cannot be saved without a category on this build, so the no-category path cannot be produced</t>
+          <t>needs a second sign-in as a user with no reports access</t>
         </is>
       </c>
       <c r="G83" s="6" t="inlineStr">
@@ -3965,22 +3989,22 @@
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>C30577</t>
+          <t>C30605</t>
         </is>
       </c>
       <c r="D84" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30577</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30605</t>
         </is>
       </c>
       <c r="E84" s="6" t="inlineStr">
         <is>
-          <t>Inventory Value: the Location filter is hidden for a one-location user</t>
+          <t>Nightly snapshot records one row per in-stock non-core part per location</t>
         </is>
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>needs a second sign-in as a user with access to only one location</t>
+          <t>the nightly capture is a server-side job and its stored rows are not reachable from the application</t>
         </is>
       </c>
       <c r="G84" s="6" t="inlineStr">
@@ -4000,22 +4024,22 @@
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>C30603</t>
+          <t>C30606</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30603</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30606</t>
         </is>
       </c>
       <c r="E85" s="6" t="inlineStr">
         <is>
-          <t>A user with ordinary reports access can open Inventory Value</t>
+          <t>A recorded snapshot day equals what the live report showed that day</t>
         </is>
       </c>
       <c r="F85" s="6" t="inlineStr">
         <is>
-          <t>needs a second sign-in as a user holding only the ordinary reports access</t>
+          <t>needs the stored nightly capture rows, which are not reachable from the application</t>
         </is>
       </c>
       <c r="G85" s="6" t="inlineStr">
@@ -4035,22 +4059,22 @@
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>C30604</t>
+          <t>C30607</t>
         </is>
       </c>
       <c r="D86" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30604</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30607</t>
         </is>
       </c>
       <c r="E86" s="6" t="inlineStr">
         <is>
-          <t>Without reports access Inventory Value is absent from the navigation</t>
+          <t>Nightly snapshot: re-running the capture for a date replaces that date's rows</t>
         </is>
       </c>
       <c r="F86" s="6" t="inlineStr">
         <is>
-          <t>needs a second sign-in as a user with no reports access</t>
+          <t>the nightly capture job cannot be re-run or inspected from the application</t>
         </is>
       </c>
       <c r="G86" s="6" t="inlineStr">
@@ -4070,22 +4094,22 @@
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>C30605</t>
+          <t>C30609</t>
         </is>
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30605</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30609</t>
         </is>
       </c>
       <c r="E87" s="6" t="inlineStr">
         <is>
-          <t>Nightly snapshot records one row per in-stock non-core part per location</t>
+          <t>Snapshot retention: daily captures are kept for 0–13 months</t>
         </is>
       </c>
       <c r="F87" s="6" t="inlineStr">
         <is>
-          <t>the nightly capture is a server-side job and its stored rows are not reachable from the application</t>
+          <t>retention pruning is a server-side job over stored history, not reachable from the application</t>
         </is>
       </c>
       <c r="G87" s="6" t="inlineStr">
@@ -4105,22 +4129,22 @@
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>C30606</t>
+          <t>C30610</t>
         </is>
       </c>
       <c r="D88" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30606</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30610</t>
         </is>
       </c>
       <c r="E88" s="6" t="inlineStr">
         <is>
-          <t>A recorded snapshot day equals what the live report showed that day</t>
+          <t>Thinned history still served by the closest-recorded-day rule</t>
         </is>
       </c>
       <c r="F88" s="6" t="inlineStr">
         <is>
-          <t>needs the stored nightly capture rows, which are not reachable from the application</t>
+          <t>needs a thinned history that this organisation does not have and cannot be produced from the application</t>
         </is>
       </c>
       <c r="G88" s="6" t="inlineStr">
@@ -4140,27 +4164,27 @@
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>C30607</t>
+          <t>C38892</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30607</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/38892</t>
         </is>
       </c>
       <c r="E89" s="6" t="inlineStr">
         <is>
-          <t>Nightly snapshot: re-running the capture for a date replaces that date's rows</t>
+          <t>A recorded day keeps its category and vendor names after a rename or delete</t>
         </is>
       </c>
       <c r="F89" s="6" t="inlineStr">
         <is>
-          <t>the nightly capture job cannot be re-run or inspected from the application</t>
+          <t>needs a recorded earlier day plus the stored capture rows, which are not reachable from the application</t>
         </is>
       </c>
       <c r="G89" s="6" t="inlineStr">
         <is>
-          <t>Untested</t>
+          <t>no result recorded — leave it, or mark Blocked</t>
         </is>
       </c>
     </row>
@@ -4175,27 +4199,27 @@
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>C30609</t>
+          <t>C38912</t>
         </is>
       </c>
       <c r="D90" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30609</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/38912</t>
         </is>
       </c>
       <c r="E90" s="6" t="inlineStr">
         <is>
-          <t>Snapshot retention: daily captures are kept for 0–13 months</t>
+          <t>Location column: shown to any multi-location user, Multiple on aggregating rows</t>
         </is>
       </c>
       <c r="F90" s="6" t="inlineStr">
         <is>
-          <t>retention pruning is a server-side job over stored history, not reachable from the application</t>
+          <t>the build does not follow the ratified Location rule; the defect is written up in DEFECTS-FOR-PERMISSION.md and needs the QA lead's permission before a ticket exists to point at</t>
         </is>
       </c>
       <c r="G90" s="6" t="inlineStr">
         <is>
-          <t>Untested</t>
+          <t>no result recorded — leave it, or mark Blocked</t>
         </is>
       </c>
     </row>
@@ -4210,27 +4234,27 @@
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>C30610</t>
+          <t>C38918</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30610</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/38918</t>
         </is>
       </c>
       <c r="E91" s="6" t="inlineStr">
         <is>
-          <t>Thinned history still served by the closest-recorded-day rule</t>
+          <t>An over-cap Work In Progress download is refused with the too-large message</t>
         </is>
       </c>
       <c r="F91" s="6" t="inlineStr">
         <is>
-          <t>needs a thinned history that this organisation does not have and cannot be produced from the application</t>
+          <t>the over-size refusal cannot be produced on this environment; no tab comes near the size limit</t>
         </is>
       </c>
       <c r="G91" s="6" t="inlineStr">
         <is>
-          <t>Untested</t>
+          <t>no result recorded — leave it, or mark Blocked</t>
         </is>
       </c>
     </row>
@@ -4245,22 +4269,22 @@
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>C38892</t>
+          <t>C43551</t>
         </is>
       </c>
       <c r="D92" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/38892</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/43551</t>
         </is>
       </c>
       <c r="E92" s="6" t="inlineStr">
         <is>
-          <t>A recorded day keeps its category and vendor names after a rename or delete</t>
+          <t>A hand-made Location column choice is remembered like any other column</t>
         </is>
       </c>
       <c r="F92" s="6" t="inlineStr">
         <is>
-          <t>needs a recorded earlier day plus the stored capture rows, which are not reachable from the application</t>
+          <t>the build does not follow the ratified Location rule; the defect is written up in DEFECTS-FOR-PERMISSION.md and needs the QA lead's permission before a ticket exists to point at</t>
         </is>
       </c>
       <c r="G92" s="6" t="inlineStr">
@@ -4280,22 +4304,22 @@
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>C38912</t>
+          <t>C43553</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/38912</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/43553</t>
         </is>
       </c>
       <c r="E93" s="6" t="inlineStr">
         <is>
-          <t>Location column: shown to any multi-location user, Multiple on aggregating rows</t>
+          <t>A logo that is set but will not load falls back to the ShopView logo</t>
         </is>
       </c>
       <c r="F93" s="6" t="inlineStr">
         <is>
-          <t>the build does not follow the ratified Location rule; the defect is written up in DEFECTS-FOR-PERMISSION.md and needs the QA lead's permission before a ticket exists to point at</t>
+          <t>this organisation has a logo that loads correctly, so the set-but-will-not-load fallback cannot be produced</t>
         </is>
       </c>
       <c r="G93" s="6" t="inlineStr">
@@ -4315,22 +4339,22 @@
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>C38918</t>
+          <t>C43558</t>
         </is>
       </c>
       <c r="D94" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/38918</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/43558</t>
         </is>
       </c>
       <c r="E94" s="6" t="inlineStr">
         <is>
-          <t>An over-cap Work In Progress download is refused with the too-large message</t>
+          <t>You cannot reach an invoice you have no permission to open</t>
         </is>
       </c>
       <c r="F94" s="6" t="inlineStr">
         <is>
-          <t>the over-size refusal cannot be produced on this environment; no tab comes near the size limit</t>
+          <t>waiting on one answer from the product owner about what the invoice number should look like, and it needs a second sign-in that cannot open work orders or part sales</t>
         </is>
       </c>
       <c r="G94" s="6" t="inlineStr">
@@ -4350,130 +4374,25 @@
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>C43551</t>
+          <t>C43559</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/43551</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/43559</t>
         </is>
       </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
-          <t>A hand-made Location column choice is remembered like any other column</t>
+          <t>Invoice # and customer name when you cannot open what they point at</t>
         </is>
       </c>
       <c r="F95" s="6" t="inlineStr">
         <is>
-          <t>the build does not follow the ratified Location rule; the defect is written up in DEFECTS-FOR-PERMISSION.md and needs the QA lead's permission before a ticket exists to point at</t>
+          <t>waiting on one answer from the product owner about what these two values should look like, and it needs a second sign-in that cannot open work orders, part sales or customers</t>
         </is>
       </c>
       <c r="G95" s="6" t="inlineStr">
-        <is>
-          <t>no result recorded — leave it, or mark Blocked</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="46" customHeight="1">
-      <c r="A96" s="6" t="n">
-        <v>89</v>
-      </c>
-      <c r="B96" s="6" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C96" s="6" t="inlineStr">
-        <is>
-          <t>C43553</t>
-        </is>
-      </c>
-      <c r="D96" s="6" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/43553</t>
-        </is>
-      </c>
-      <c r="E96" s="6" t="inlineStr">
-        <is>
-          <t>A logo that is set but will not load falls back to the ShopView logo</t>
-        </is>
-      </c>
-      <c r="F96" s="6" t="inlineStr">
-        <is>
-          <t>this organisation has a logo that loads correctly, so the set-but-will-not-load fallback cannot be produced</t>
-        </is>
-      </c>
-      <c r="G96" s="6" t="inlineStr">
-        <is>
-          <t>no result recorded — leave it, or mark Blocked</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="46" customHeight="1">
-      <c r="A97" s="6" t="n">
-        <v>90</v>
-      </c>
-      <c r="B97" s="6" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C97" s="6" t="inlineStr">
-        <is>
-          <t>C43558</t>
-        </is>
-      </c>
-      <c r="D97" s="6" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/43558</t>
-        </is>
-      </c>
-      <c r="E97" s="6" t="inlineStr">
-        <is>
-          <t>You cannot reach an invoice you have no permission to open</t>
-        </is>
-      </c>
-      <c r="F97" s="6" t="inlineStr">
-        <is>
-          <t>waiting on one answer from the product owner about what the invoice number should look like, and it needs a second sign-in that cannot open work orders or part sales</t>
-        </is>
-      </c>
-      <c r="G97" s="6" t="inlineStr">
-        <is>
-          <t>no result recorded — leave it, or mark Blocked</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="46" customHeight="1">
-      <c r="A98" s="6" t="n">
-        <v>91</v>
-      </c>
-      <c r="B98" s="6" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C98" s="6" t="inlineStr">
-        <is>
-          <t>C43559</t>
-        </is>
-      </c>
-      <c r="D98" s="6" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/43559</t>
-        </is>
-      </c>
-      <c r="E98" s="6" t="inlineStr">
-        <is>
-          <t>Invoice # and customer name when you cannot open what they point at</t>
-        </is>
-      </c>
-      <c r="F98" s="6" t="inlineStr">
-        <is>
-          <t>waiting on one answer from the product owner about what these two values should look like, and it needs a second sign-in that cannot open work orders, part sales or customers</t>
-        </is>
-      </c>
-      <c r="G98" s="6" t="inlineStr">
         <is>
           <t>no result recorded — leave it, or mark Blocked</t>
         </is>

</xml_diff>